<commit_message>
Suppression de la charge horaire des autonomies
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucbr\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucbr\OneDrive\Documents\GitHub\RTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA89E348-A66E-4594-8777-F9F5BBB7AA18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F3E40D8-056E-4B96-95D8-65A0390F072A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -477,7 +477,7 @@
         <v>15</v>
       </c>
       <c r="D8" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="4"/>
     </row>
@@ -492,7 +492,7 @@
         <v>17</v>
       </c>
       <c r="D9" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
ajout du projet des algos
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucbr\OneDrive\Documents\GitHub\RTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E81AFA2D-E40F-491B-B5A6-6E4D8C506881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{900958F4-5A88-4B0B-BCD2-A6C1B914384D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3945" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
   <si>
     <t>Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -97,18 +97,34 @@
     <t>Exercices partie 2</t>
   </si>
   <si>
-    <t>Début du multi-agent proie</t>
+    <t>15/09/26 - 8h30/12h30</t>
+  </si>
+  <si>
+    <t>Multi-agent proie</t>
+  </si>
+  <si>
+    <t>Début des algos</t>
+  </si>
+  <si>
+    <t>Début rencontres</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -180,21 +196,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -418,7 +435,7 @@
     <col min="2" max="2" width="47.140625" customWidth="1"/>
     <col min="3" max="3" width="16.85546875" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
     <col min="6" max="8" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -531,7 +548,7 @@
         <v>23</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>17</v>
@@ -540,7 +557,39 @@
         <v>2</v>
       </c>
     </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="6">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>27</v>
+      </c>
+    </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="6">
+        <v>2</v>
+      </c>
+      <c r="E13" t="s">
+        <v>28</v>
+      </c>
       <c r="G13" s="4"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
ajout des algorithmes des exercices 2
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucbr\OneDrive\Documents\GitHub\RTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{900958F4-5A88-4B0B-BCD2-A6C1B914384D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D19A1398-1BFF-48FB-BF42-73C3E47C0EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3945" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
   <si>
     <t>Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -107,17 +120,36 @@
   </si>
   <si>
     <t>Début rencontres</t>
+  </si>
+  <si>
+    <t>15/09/26 - 10h30/11h30</t>
+  </si>
+  <si>
+    <t>Algorithmes exercices 2.5</t>
+  </si>
+  <si>
+    <t>Héritage des objets proies</t>
+  </si>
+  <si>
+    <t>jusqu'au 2.3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -196,21 +228,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -542,6 +575,9 @@
       <c r="D10" s="6">
         <v>2</v>
       </c>
+      <c r="E10" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
@@ -593,7 +629,33 @@
       <c r="G13" s="4"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="6">
+        <v>0</v>
+      </c>
       <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">

</xml_diff>

<commit_message>
Implémentation du Lotka Volterra semi implicite
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucbr\OneDrive\Documents\GitHub\RTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D19A1398-1BFF-48FB-BF42-73C3E47C0EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC5D617-C7C0-455D-ACC8-E075E2F12B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="42">
   <si>
     <t>Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -132,17 +132,51 @@
   </si>
   <si>
     <t>jusqu'au 2.3</t>
+  </si>
+  <si>
+    <t>17/09/26 - 10h30/12h30</t>
+  </si>
+  <si>
+    <t>Algorithmes  + exercices 2.6</t>
+  </si>
+  <si>
+    <t>Reproduction par rencontres et âges</t>
+  </si>
+  <si>
+    <t>17/09/26 - 13h45/15h45</t>
+  </si>
+  <si>
+    <t>Exercice 2.7</t>
+  </si>
+  <si>
+    <t>Multi agent prédateur début</t>
+  </si>
+  <si>
+    <t>Multi-agent proie début</t>
+  </si>
+  <si>
+    <t>Début Lotka Volterra implicite</t>
+  </si>
+  <si>
+    <t>forme semi-implicite</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -228,21 +262,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -468,7 +503,7 @@
     <col min="2" max="2" width="47.140625" customWidth="1"/>
     <col min="3" max="3" width="16.85546875" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" customWidth="1"/>
     <col min="6" max="8" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -615,7 +650,7 @@
         <v>25</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>17</v>
@@ -657,27 +692,100 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="6">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="E20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Mis à jour des tâches
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucbr\OneDrive\Documents\GitHub\RTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC5D617-C7C0-455D-ACC8-E075E2F12B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17EB9984-57F6-4EB6-816E-0045D37DED1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3945" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="46">
   <si>
     <t>Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -159,17 +159,36 @@
   </si>
   <si>
     <t>forme semi-implicite</t>
+  </si>
+  <si>
+    <t>21/09/26 - 10h30/12h30</t>
+  </si>
+  <si>
+    <t>Lotka Volterra semi-implicite</t>
+  </si>
+  <si>
+    <t>algorithme</t>
+  </si>
+  <si>
+    <t>Optimisation des performances</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -262,21 +281,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -765,6 +785,37 @@
         <v>41</v>
       </c>
     </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="6">
+        <v>1</v>
+      </c>
+      <c r="E21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22" s="6">
+        <v>2</v>
+      </c>
+    </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Ajout des vérifications des exercices
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucbr\OneDrive\Documents\GitHub\RTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17EB9984-57F6-4EB6-816E-0045D37DED1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547F3BF0-FD14-4912-8934-D0AD4F6157F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3945" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="48">
   <si>
     <t>Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -171,6 +171,12 @@
   </si>
   <si>
     <t>Optimisation des performances</t>
+  </si>
+  <si>
+    <t>Début exercices 3</t>
+  </si>
+  <si>
+    <t>3.1</t>
   </si>
 </sst>
 </file>
@@ -816,6 +822,23 @@
         <v>2</v>
       </c>
     </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="6">
+        <v>1</v>
+      </c>
+      <c r="E23" t="s">
+        <v>47</v>
+      </c>
+    </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
mise à jour des tâches et ajout des diagrammes 3.2 et 3.3
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucbr\OneDrive\Documents\GitHub\RTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA0869B-E0D1-4EAC-85BF-1732915B88FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8E218E-6826-4C8E-8930-698AEF0E5216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="64">
   <si>
     <t>Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -198,6 +198,33 @@
   </si>
   <si>
     <t>Rencontre des prédateurs</t>
+  </si>
+  <si>
+    <t>23/09/26 - 13h45/15h45</t>
+  </si>
+  <si>
+    <t>23/09/26 - 16h/18h</t>
+  </si>
+  <si>
+    <t>Fin exercices 3.2</t>
+  </si>
+  <si>
+    <t>Fin rencontre des prédateurs</t>
+  </si>
+  <si>
+    <t>Début exercices 3.3</t>
+  </si>
+  <si>
+    <t>Début couplage proie/prédateur</t>
+  </si>
+  <si>
+    <t>Fin exercice 3.3</t>
+  </si>
+  <si>
+    <t>Début exercice 3.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Couplage proie/prédateur </t>
   </si>
 </sst>
 </file>
@@ -315,43 +342,6 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
         <color rgb="FFFF0000"/>
         <name val="Calibri"/>
         <family val="2"/>
@@ -390,6 +380,43 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Calibri"/>
         <scheme val="minor"/>
@@ -409,13 +436,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63278AAA-70E1-41D7-BAA0-A60274FB135D}" name="Tableau1" displayName="Tableau1" ref="B5:F27" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="B5:F27" xr:uid="{63278AAA-70E1-41D7-BAA0-A60274FB135D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63278AAA-70E1-41D7-BAA0-A60274FB135D}" name="Tableau1" displayName="Tableau1" ref="B5:F35" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="B5:F35" xr:uid="{63278AAA-70E1-41D7-BAA0-A60274FB135D}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{06615344-F11A-476A-9717-0137331FFCD4}" name="Séance :" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{6BDB3C24-9120-4506-AC41-7C407DF8AE42}" name="Tâche réalisée :" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{E6006A89-3B13-4E71-B0C8-0AB1DF00D794}" name="Etudiant :" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{AA5A3BE2-FE7E-45DB-9B0C-2FD69D27DE6A}" name="Charge retenue (h) :" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{06615344-F11A-476A-9717-0137331FFCD4}" name="Séance :" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{6BDB3C24-9120-4506-AC41-7C407DF8AE42}" name="Tâche réalisée :" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{E6006A89-3B13-4E71-B0C8-0AB1DF00D794}" name="Etudiant :" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{AA5A3BE2-FE7E-45DB-9B0C-2FD69D27DE6A}" name="Charge retenue (h) :" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{3FD5E7F7-5EC0-435B-8103-AB9356B2E2BD}" name="Commentaires :"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -620,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
@@ -1019,6 +1046,113 @@
         <v>48</v>
       </c>
     </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" s="7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="7">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B32" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B34" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" s="7">
+        <v>1</v>
+      </c>
+      <c r="F34" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="8"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="7"/>
+    </row>
   </sheetData>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>